<commit_message>
fix: update error message and instructions for data entry in StudentImportModal
</commit_message>
<xml_diff>
--- a/public/templates/template_biodata_siswa.xlsx
+++ b/public/templates/template_biodata_siswa.xlsx
@@ -686,223 +686,223 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>12345</v>
+      </c>
+      <c r="B8" t="str">
+        <v>X TJKT 1</v>
+      </c>
+      <c r="C8" t="str">
+        <v>0061234567</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Teknik Komputer dan Jaringan (TJKT)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Ahmad Fauzi</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Fauzi</v>
+      </c>
+      <c r="G8" t="str">
+        <v>L</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Tangerang</v>
+      </c>
+      <c r="I8" t="str">
+        <v>17/08/2006</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Islam</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Indonesia</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2</v>
+      </c>
+      <c r="M8" t="str">
+        <v>2</v>
+      </c>
+      <c r="N8" t="str">
         <v>1</v>
       </c>
-      <c r="B8" t="str">
-        <v>2</v>
-      </c>
-      <c r="C8" t="str">
-        <v>3</v>
-      </c>
-      <c r="D8" t="str">
-        <v>4</v>
-      </c>
-      <c r="E8" t="str">
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v>Indonesia</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Jl. Raya Serpong No. 12, Kelapa Dua</v>
+      </c>
+      <c r="R8" t="str">
+        <v>081234567890</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Orang Tua</v>
+      </c>
+      <c r="T8" t="str">
         <v>5</v>
       </c>
-      <c r="F8" t="str">
+      <c r="U8" t="str">
+        <v>O</v>
+      </c>
+      <c r="V8" t="str">
+        <v>-</v>
+      </c>
+      <c r="W8" t="str">
+        <v>-</v>
+      </c>
+      <c r="X8" t="str">
+        <v>170</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>58</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>SMPN 1 Tangerang</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>10/06/2021</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>DN-06-Dd-2021-0001234</v>
+      </c>
+      <c r="AC8" t="str">
         <v>6</v>
       </c>
-      <c r="G8" t="str">
-        <v>7</v>
-      </c>
-      <c r="H8" t="str">
-        <v>8</v>
-      </c>
-      <c r="I8" t="str">
-        <v>9</v>
-      </c>
-      <c r="J8" t="str">
-        <v>10</v>
-      </c>
-      <c r="K8" t="str">
-        <v>11</v>
-      </c>
-      <c r="L8" t="str">
-        <v>12</v>
-      </c>
-      <c r="M8" t="str">
-        <v>13</v>
-      </c>
-      <c r="N8" t="str">
-        <v>14</v>
-      </c>
-      <c r="O8" t="str">
-        <v>15</v>
-      </c>
-      <c r="P8" t="str">
-        <v>16</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>17</v>
-      </c>
-      <c r="R8" t="str">
-        <v>18</v>
-      </c>
-      <c r="S8" t="str">
-        <v>19</v>
-      </c>
-      <c r="T8" t="str">
-        <v>20</v>
-      </c>
-      <c r="U8" t="str">
-        <v>21</v>
-      </c>
-      <c r="V8" t="str">
-        <v>22</v>
-      </c>
-      <c r="W8" t="str">
-        <v>23</v>
-      </c>
-      <c r="X8" t="str">
-        <v>24</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>25</v>
-      </c>
-      <c r="Z8" t="str">
-        <v>26</v>
-      </c>
-      <c r="AA8" t="str">
-        <v>27</v>
-      </c>
-      <c r="AB8" t="str">
-        <v>28</v>
-      </c>
-      <c r="AC8" t="str">
-        <v>29</v>
-      </c>
       <c r="AD8" t="str">
-        <v>30</v>
+        <v/>
       </c>
       <c r="AE8" t="str">
-        <v>31</v>
+        <v/>
       </c>
       <c r="AF8" t="str">
-        <v>32</v>
+        <v/>
       </c>
       <c r="AG8" t="str">
-        <v>33</v>
+        <v/>
       </c>
       <c r="AH8" t="str">
-        <v>34</v>
+        <v>15/07/2021</v>
       </c>
       <c r="AI8" t="str">
-        <v>35</v>
+        <v>Budi Santoso</v>
       </c>
       <c r="AJ8" t="str">
-        <v>36</v>
+        <v>Tangerang</v>
       </c>
       <c r="AK8" t="str">
-        <v>37</v>
+        <v>01/01/1978</v>
       </c>
       <c r="AL8" t="str">
-        <v>38</v>
+        <v>Islam</v>
       </c>
       <c r="AM8" t="str">
-        <v>39</v>
+        <v>Indonesia</v>
       </c>
       <c r="AN8" t="str">
-        <v>40</v>
+        <v>SMA</v>
       </c>
       <c r="AO8" t="str">
-        <v>41</v>
+        <v>Wiraswasta</v>
       </c>
       <c r="AP8" t="str">
-        <v>42</v>
+        <v>3000000</v>
       </c>
       <c r="AQ8" t="str">
-        <v>43</v>
+        <v>Jl. Raya Serpong No. 12</v>
       </c>
       <c r="AR8" t="str">
-        <v>44</v>
+        <v>081234567891</v>
       </c>
       <c r="AS8" t="str">
-        <v>45</v>
+        <v>Masih Hidup</v>
       </c>
       <c r="AT8" t="str">
-        <v>46</v>
+        <v>Siti Rahayu</v>
       </c>
       <c r="AU8" t="str">
-        <v>47</v>
+        <v>Tangerang</v>
       </c>
       <c r="AV8" t="str">
-        <v>48</v>
+        <v>15/03/1980</v>
       </c>
       <c r="AW8" t="str">
-        <v>49</v>
+        <v>Islam</v>
       </c>
       <c r="AX8" t="str">
-        <v>50</v>
+        <v>Indonesia</v>
       </c>
       <c r="AY8" t="str">
-        <v>51</v>
+        <v>SMA</v>
       </c>
       <c r="AZ8" t="str">
-        <v>52</v>
+        <v>Ibu Rumah Tangga</v>
       </c>
       <c r="BA8" t="str">
-        <v>53</v>
+        <v>-</v>
       </c>
       <c r="BB8" t="str">
-        <v>54</v>
+        <v>Jl. Raya Serpong No. 12</v>
       </c>
       <c r="BC8" t="str">
-        <v>55</v>
+        <v>081234567892</v>
       </c>
       <c r="BD8" t="str">
-        <v>56</v>
+        <v>Masih Hidup</v>
       </c>
       <c r="BE8" t="str">
-        <v>57</v>
+        <v>Budi Santoso</v>
       </c>
       <c r="BF8" t="str">
-        <v>58</v>
+        <v>Tangerang</v>
       </c>
       <c r="BG8" t="str">
-        <v>59</v>
+        <v>01/01/1978</v>
       </c>
       <c r="BH8" t="str">
-        <v>60</v>
+        <v>Islam</v>
       </c>
       <c r="BI8" t="str">
-        <v>61</v>
+        <v>Indonesia</v>
       </c>
       <c r="BJ8" t="str">
-        <v>62</v>
+        <v>SMA</v>
       </c>
       <c r="BK8" t="str">
-        <v>63</v>
+        <v>Wiraswasta</v>
       </c>
       <c r="BL8" t="str">
-        <v>64</v>
+        <v>3000000</v>
       </c>
       <c r="BM8" t="str">
-        <v>65</v>
+        <v>Jl. Raya Serpong No. 12</v>
       </c>
       <c r="BN8" t="str">
-        <v>66</v>
+        <v>081234567891</v>
       </c>
       <c r="BO8" t="str">
-        <v>67</v>
+        <v>Menggambar</v>
       </c>
       <c r="BP8" t="str">
-        <v>68</v>
+        <v>Bulu Tangkis</v>
       </c>
       <c r="BQ8" t="str">
-        <v>69</v>
+        <v>Karang Taruna</v>
       </c>
       <c r="BR8" t="str">
-        <v>70</v>
+        <v/>
       </c>
       <c r="BS8" t="str">
-        <v>71</v>
+        <v>Peserta Didik</v>
       </c>
       <c r="BT8" t="str">
-        <v>72</v>
+        <v>15/07/2021</v>
       </c>
       <c r="BU8" t="str">
-        <v>73</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update student biodata to support decimal type for distance and enhance input handling
</commit_message>
<xml_diff>
--- a/public/templates/template_biodata_siswa.xlsx
+++ b/public/templates/template_biodata_siswa.xlsx
@@ -686,94 +686,94 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>1</v>
+      </c>
+      <c r="B8" t="str">
         <v>12345</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>X TJKT 1</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>0061234567</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Teknik Komputer dan Jaringan (TJKT)</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Ahmad Fauzi</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Fauzi</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>L</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>Tangerang</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>17/08/2006</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>Islam</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Indonesia</v>
-      </c>
-      <c r="L8" t="str">
-        <v>2</v>
       </c>
       <c r="M8" t="str">
         <v>2</v>
       </c>
       <c r="N8" t="str">
+        <v>2</v>
+      </c>
+      <c r="O8" t="str">
         <v>1</v>
       </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
         <v/>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>Indonesia</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="R8" t="str">
         <v>Jl. Raya Serpong No. 12, Kelapa Dua</v>
       </c>
-      <c r="R8" t="str">
+      <c r="S8" t="str">
         <v>081234567890</v>
       </c>
-      <c r="S8" t="str">
+      <c r="T8" t="str">
         <v>Orang Tua</v>
       </c>
-      <c r="T8" t="str">
+      <c r="U8" t="str">
         <v>5</v>
       </c>
-      <c r="U8" t="str">
+      <c r="V8" t="str">
         <v>O</v>
-      </c>
-      <c r="V8" t="str">
-        <v>-</v>
       </c>
       <c r="W8" t="str">
         <v>-</v>
       </c>
       <c r="X8" t="str">
+        <v>-</v>
+      </c>
+      <c r="Y8" t="str">
         <v>170</v>
       </c>
-      <c r="Y8" t="str">
+      <c r="Z8" t="str">
         <v>58</v>
       </c>
-      <c r="Z8" t="str">
+      <c r="AA8" t="str">
         <v>SMPN 1 Tangerang</v>
       </c>
-      <c r="AA8" t="str">
+      <c r="AB8" t="str">
         <v>10/06/2021</v>
       </c>
-      <c r="AB8" t="str">
+      <c r="AC8" t="str">
         <v>DN-06-Dd-2021-0001234</v>
       </c>
-      <c r="AC8" t="str">
+      <c r="AD8" t="str">
         <v>6</v>
-      </c>
-      <c r="AD8" t="str">
-        <v/>
       </c>
       <c r="AE8" t="str">
         <v/>
@@ -785,124 +785,124 @@
         <v/>
       </c>
       <c r="AH8" t="str">
+        <v/>
+      </c>
+      <c r="AI8" t="str">
         <v>15/07/2021</v>
       </c>
-      <c r="AI8" t="str">
+      <c r="AJ8" t="str">
         <v>Budi Santoso</v>
       </c>
-      <c r="AJ8" t="str">
+      <c r="AK8" t="str">
         <v>Tangerang</v>
       </c>
-      <c r="AK8" t="str">
+      <c r="AL8" t="str">
         <v>01/01/1978</v>
       </c>
-      <c r="AL8" t="str">
+      <c r="AM8" t="str">
         <v>Islam</v>
       </c>
-      <c r="AM8" t="str">
+      <c r="AN8" t="str">
         <v>Indonesia</v>
       </c>
-      <c r="AN8" t="str">
+      <c r="AO8" t="str">
         <v>SMA</v>
       </c>
-      <c r="AO8" t="str">
+      <c r="AP8" t="str">
         <v>Wiraswasta</v>
       </c>
-      <c r="AP8" t="str">
+      <c r="AQ8" t="str">
         <v>3000000</v>
       </c>
-      <c r="AQ8" t="str">
+      <c r="AR8" t="str">
         <v>Jl. Raya Serpong No. 12</v>
       </c>
-      <c r="AR8" t="str">
+      <c r="AS8" t="str">
         <v>081234567891</v>
       </c>
-      <c r="AS8" t="str">
+      <c r="AT8" t="str">
         <v>Masih Hidup</v>
       </c>
-      <c r="AT8" t="str">
+      <c r="AU8" t="str">
         <v>Siti Rahayu</v>
       </c>
-      <c r="AU8" t="str">
+      <c r="AV8" t="str">
         <v>Tangerang</v>
       </c>
-      <c r="AV8" t="str">
+      <c r="AW8" t="str">
         <v>15/03/1980</v>
       </c>
-      <c r="AW8" t="str">
+      <c r="AX8" t="str">
         <v>Islam</v>
       </c>
-      <c r="AX8" t="str">
+      <c r="AY8" t="str">
         <v>Indonesia</v>
       </c>
-      <c r="AY8" t="str">
+      <c r="AZ8" t="str">
         <v>SMA</v>
       </c>
-      <c r="AZ8" t="str">
+      <c r="BA8" t="str">
         <v>Ibu Rumah Tangga</v>
       </c>
-      <c r="BA8" t="str">
+      <c r="BB8" t="str">
         <v>-</v>
       </c>
-      <c r="BB8" t="str">
+      <c r="BC8" t="str">
         <v>Jl. Raya Serpong No. 12</v>
       </c>
-      <c r="BC8" t="str">
+      <c r="BD8" t="str">
         <v>081234567892</v>
       </c>
-      <c r="BD8" t="str">
+      <c r="BE8" t="str">
         <v>Masih Hidup</v>
       </c>
-      <c r="BE8" t="str">
+      <c r="BF8" t="str">
         <v>Budi Santoso</v>
       </c>
-      <c r="BF8" t="str">
+      <c r="BG8" t="str">
         <v>Tangerang</v>
       </c>
-      <c r="BG8" t="str">
+      <c r="BH8" t="str">
         <v>01/01/1978</v>
       </c>
-      <c r="BH8" t="str">
+      <c r="BI8" t="str">
         <v>Islam</v>
       </c>
-      <c r="BI8" t="str">
+      <c r="BJ8" t="str">
         <v>Indonesia</v>
       </c>
-      <c r="BJ8" t="str">
+      <c r="BK8" t="str">
         <v>SMA</v>
       </c>
-      <c r="BK8" t="str">
+      <c r="BL8" t="str">
         <v>Wiraswasta</v>
       </c>
-      <c r="BL8" t="str">
+      <c r="BM8" t="str">
         <v>3000000</v>
       </c>
-      <c r="BM8" t="str">
+      <c r="BN8" t="str">
         <v>Jl. Raya Serpong No. 12</v>
       </c>
-      <c r="BN8" t="str">
+      <c r="BO8" t="str">
         <v>081234567891</v>
       </c>
-      <c r="BO8" t="str">
+      <c r="BP8" t="str">
         <v>Menggambar</v>
       </c>
-      <c r="BP8" t="str">
+      <c r="BQ8" t="str">
         <v>Bulu Tangkis</v>
       </c>
-      <c r="BQ8" t="str">
+      <c r="BR8" t="str">
         <v>Karang Taruna</v>
       </c>
-      <c r="BR8" t="str">
+      <c r="BS8" t="str">
         <v/>
       </c>
-      <c r="BS8" t="str">
+      <c r="BT8" t="str">
         <v>Peserta Didik</v>
       </c>
-      <c r="BT8" t="str">
+      <c r="BU8" t="str">
         <v>15/07/2021</v>
-      </c>
-      <c r="BU8" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add class validation and normalization for student records
</commit_message>
<xml_diff>
--- a/public/templates/template_biodata_siswa.xlsx
+++ b/public/templates/template_biodata_siswa.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Petunjuk Penggunaan" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -122,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -157,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -404,6 +405,9 @@
       <c r="A1" t="str">
         <v>BIODATA PESERTA DIDIK BARU</v>
       </c>
+      <c r="U1" t="str">
+        <v>PETUNJUK PENGGUNAAN: lihat sheet "Petunjuk Penggunaan" sebelum mengisi template.</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -692,13 +696,13 @@
         <v>12345</v>
       </c>
       <c r="C8" t="str">
-        <v>X TJKT 1</v>
+        <v>XI</v>
       </c>
       <c r="D8" t="str">
         <v>0061234567</v>
       </c>
       <c r="E8" t="str">
-        <v>Teknik Komputer dan Jaringan (TJKT)</v>
+        <v>TJKT</v>
       </c>
       <c r="F8" t="str">
         <v>Ahmad Fauzi</v>
@@ -906,7 +910,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="86">
+  <mergeCells count="87">
     <mergeCell ref="BT6:BT7"/>
     <mergeCell ref="BU6:BU7"/>
     <mergeCell ref="BP6:BP7"/>
@@ -993,10 +997,153 @@
     <mergeCell ref="A4:Q4"/>
     <mergeCell ref="R4:U4"/>
     <mergeCell ref="V4:Z4"/>
+    <mergeCell ref="U1:BU1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:BU8"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A25"/>
+  <cols>
+    <col min="1" max="1" width="105.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PETUNJUK PENGGUNAAN TEMPLATE BIODATA SISWA</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Template ini dipakai pada menu Data Siswa &gt; Import Excel. Ikuti aturan berikut:</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A. STRUKTUR TEMPLATE</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>1. Sheet1 berisi header 3 lapis (baris 1-7). JANGAN mengubah/menghapus header ini.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2. Baris 8 adalah baris CONTOH dan otomatis dilewati saat import.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>3. Isi data siswa mulai BARIS 9, satu siswa per baris.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>B. ATURAN PENGISIAN</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1. Kolom WAJIB diisi: NISN dan NAMA.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2. NISN dan NIS diisi dengan format TEKS di Excel agar angka 0 di awal tidak hilang.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>3. KELAS hanya boleh X, XI, atau XII (tingkat kelas saja, bukan gabungan jurusan).</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v xml:space="preserve">   Contoh benar : XI</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">   Contoh salah : X TJKT, XI TJKT 1, 13, kelas XI</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>4. JURUSAN diisi TERPISAH pada kolom JURUSAN. Contoh: TJKT</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v xml:space="preserve">   Kelas   : XI</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">   Jurusan : TJKT</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>5. JENIS KELAMIN: isi L atau P (Laki-laki/Perempuan juga diterima).</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>6. TANGGAL menerima format DD/MM/YYYY atau YYYY-MM-DD.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>7. PIN login siswa dibuat otomatis dari 4 digit terakhir NISN.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>C. HASIL IMPORT</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Baris yang tidak valid (NISN/NIS duplikat, NISN &lt; 4 digit, Kelas tidak valid, dll.) otomatis</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>dilewati dan dicatat beserta nomor barisnya pada laporan hasil import.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A25"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>